<commit_message>
Bedrijfsadres overal Driemanssteeweg 412, 3084 CB Rotterdam (was Arnhemseweg 12 Barendrecht), ondertekenplaats Rotterdam; vangnet: instellingen nooit volledig leeg opslaan
</commit_message>
<xml_diff>
--- a/public/templates/evaluaties/Q4S B.V.-VG-evaluatieformulier door inlener(VCU) (1).xlsx
+++ b/public/templates/evaluaties/Q4S B.V.-VG-evaluatieformulier door inlener(VCU) (1).xlsx
@@ -68,10 +68,10 @@
     <t>Q4S B.V.</t>
   </si>
   <si>
-    <t>Arnhemseweg 12 2994LA</t>
-  </si>
-  <si>
-    <t>Barendrecht</t>
+    <t>Driemanssteeweg 412 3084 CB</t>
+  </si>
+  <si>
+    <t>Rotterdam</t>
   </si>
   <si>
     <t>Evaluatie door inleenbedrijf over uitzendkracht</t>

</xml_diff>